<commit_message>
11/8/2023 11:20 AM commit
</commit_message>
<xml_diff>
--- a/SFN/ACC activation mask/iosXacc(model2).xlsx
+++ b/SFN/ACC activation mask/iosXacc(model2).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/avidachs/Documents/GitHub/rf1-sra-trust/SFN/ACC activation mask/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D39B8CFA-CF6A-9845-909C-067539E245C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{316EB3B8-BE1B-BA48-9C89-B78380D0409C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7180" yWindow="2960" windowWidth="21240" windowHeight="13660" xr2:uid="{3A5DD16A-A3C8-F048-9FB6-87C8858499AB}"/>
+    <workbookView xWindow="6920" yWindow="500" windowWidth="21240" windowHeight="13660" xr2:uid="{3A5DD16A-A3C8-F048-9FB6-87C8858499AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -421,42 +421,42 @@
     </row>
     <row r="2" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
-        <v>-0.53225806499999995</v>
+        <v>-5.5322580649999997</v>
       </c>
       <c r="B2" s="2">
-        <v>76.777550529999999</v>
+        <v>-339.99307579999999</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
-        <v>-1.5322580649999999</v>
+        <v>-3.5322580650000002</v>
       </c>
       <c r="B3" s="2">
-        <v>-189.10152590000001</v>
+        <v>-282.54066890000001</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
-        <v>2.4677419349999998</v>
+        <v>-3.5322580650000002</v>
       </c>
       <c r="B4" s="2">
-        <v>-99.140508990000001</v>
+        <v>-177.84190140000001</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
-        <v>2.4677419349999998</v>
+        <v>-2.5322580650000002</v>
       </c>
       <c r="B5" s="2">
-        <v>42.346313539999997</v>
+        <v>-169.69919909999999</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
-        <v>-1.5322580649999999</v>
+        <v>-2.5322580650000002</v>
       </c>
       <c r="B6" s="2">
-        <v>-39.295127549999997</v>
+        <v>-191.7382771</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="21" x14ac:dyDescent="0.3">
@@ -464,7 +464,7 @@
         <v>-2.5322580650000002</v>
       </c>
       <c r="B7" s="2">
-        <v>-169.69919909999999</v>
+        <v>-194.48750079999999</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="21" x14ac:dyDescent="0.3">
@@ -472,231 +472,231 @@
         <v>-2.5322580650000002</v>
       </c>
       <c r="B8" s="2">
-        <v>-191.7382771</v>
+        <v>-109.4714515</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
-        <v>1.4677419350000001</v>
+        <v>-2.5322580650000002</v>
       </c>
       <c r="B9" s="2">
-        <v>392.72608220000001</v>
+        <v>-263.95745219999998</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
-        <v>2.4677419349999998</v>
+        <v>-2.5322580650000002</v>
       </c>
       <c r="B10" s="2">
-        <v>-14.619110620000001</v>
+        <v>-211.49085249999999</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
-        <v>0.467741935</v>
+        <v>-2.5322580650000002</v>
       </c>
       <c r="B11" s="2">
-        <v>-36.927186759999998</v>
+        <v>-101.92164959999999</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
-        <v>-0.53225806499999995</v>
+        <v>-2.5322580650000002</v>
       </c>
       <c r="B12" s="2">
-        <v>-187.4876999</v>
+        <v>-201.29575170000001</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
-        <v>-0.53225806499999995</v>
+        <v>-2.5322580650000002</v>
       </c>
       <c r="B13" s="2">
-        <v>326.8048814</v>
+        <v>-364.66371650000002</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
-        <v>2.4677419349999998</v>
+        <v>-1.5322580649999999</v>
       </c>
       <c r="B14" s="2">
-        <v>385.94761240000003</v>
+        <v>-189.10152590000001</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
-        <v>0.467741935</v>
+        <v>-1.5322580649999999</v>
       </c>
       <c r="B15" s="2">
-        <v>126.02746999999999</v>
+        <v>-39.295127549999997</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
-        <v>2.4677419349999998</v>
+        <v>-1.5322580649999999</v>
       </c>
       <c r="B16" s="2">
-        <v>322.39920560000002</v>
+        <v>-434.67471069999999</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
-        <v>1.4677419350000001</v>
+        <v>-1.5322580649999999</v>
       </c>
       <c r="B17" s="2">
-        <v>-215.16667810000001</v>
+        <v>43.387322150000003</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
-        <v>1.4677419350000001</v>
+        <v>-1.5322580649999999</v>
       </c>
       <c r="B18" s="2">
-        <v>-137.25841019999999</v>
+        <v>291.83634439999997</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
-        <v>-2.5322580650000002</v>
+        <v>-0.53225806499999995</v>
       </c>
       <c r="B19" s="2">
-        <v>-194.48750079999999</v>
+        <v>76.777550529999999</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
-        <v>1.4677419350000001</v>
+        <v>-0.53225806499999995</v>
       </c>
       <c r="B20" s="2">
-        <v>302.06583760000001</v>
+        <v>-187.4876999</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
-        <v>0.467741935</v>
+        <v>-0.53225806499999995</v>
       </c>
       <c r="B21" s="2">
-        <v>-24.80684389</v>
+        <v>326.8048814</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
-        <v>1.4677419350000001</v>
+        <v>-0.53225806499999995</v>
       </c>
       <c r="B22" s="2">
-        <v>383.43439669999998</v>
+        <v>117.7525231</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
-        <v>-2.5322580650000002</v>
+        <v>-0.53225806499999995</v>
       </c>
       <c r="B23" s="2">
-        <v>-109.4714515</v>
+        <v>-134.89766950000001</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
-        <v>2.4677419349999998</v>
+        <v>-0.53225806499999995</v>
       </c>
       <c r="B24" s="2">
-        <v>-197.3118254</v>
+        <v>196.89492379999999</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
-        <v>1.4677419350000001</v>
+        <v>-0.53225806499999995</v>
       </c>
       <c r="B25" s="2">
-        <v>85.329523769999994</v>
+        <v>-93.904660309999997</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
-        <v>2.4677419349999998</v>
+        <v>-0.53225806499999995</v>
       </c>
       <c r="B26" s="2">
-        <v>-143.12308340000001</v>
+        <v>120.81428390000001</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
-        <v>2.4677419349999998</v>
+        <v>-0.53225806499999995</v>
       </c>
       <c r="B27" s="2">
-        <v>209.39893910000001</v>
+        <v>-91.061769920000003</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
-        <v>2.4677419349999998</v>
+        <v>-0.53225806499999995</v>
       </c>
       <c r="B28" s="2">
-        <v>145.41335430000001</v>
+        <v>88.617453889999993</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
-        <v>2.4677419349999998</v>
+        <v>-0.53225806499999995</v>
       </c>
       <c r="B29" s="2">
-        <v>200.7153544</v>
+        <v>-59.240526150000001</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
-        <v>-2.5322580650000002</v>
+        <v>-0.53225806499999995</v>
       </c>
       <c r="B30" s="2">
-        <v>-263.95745219999998</v>
+        <v>99.439455199999998</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
-        <v>1.4677419350000001</v>
+        <v>-0.53225806499999995</v>
       </c>
       <c r="B31" s="2">
-        <v>29.76821545</v>
+        <v>252.8407685</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
-        <v>1.4677419350000001</v>
+        <v>-0.53225806499999995</v>
       </c>
       <c r="B32" s="2">
-        <v>86.447454379999996</v>
+        <v>426.76154459999998</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
-        <v>1.4677419350000001</v>
+        <v>-0.53225806499999995</v>
       </c>
       <c r="B33" s="2">
-        <v>263.80129269999998</v>
+        <v>-157.17071999999999</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
-        <v>-0.53225806499999995</v>
+        <v>0.467741935</v>
       </c>
       <c r="B34" s="2">
-        <v>117.7525231</v>
+        <v>-36.927186759999998</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
-        <v>-0.53225806499999995</v>
+        <v>0.467741935</v>
       </c>
       <c r="B35" s="2">
-        <v>-134.89766950000001</v>
+        <v>126.02746999999999</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
-        <v>1.4677419350000001</v>
+        <v>0.467741935</v>
       </c>
       <c r="B36" s="2">
-        <v>-10.90527734</v>
+        <v>-24.80684389</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="21" x14ac:dyDescent="0.3">
@@ -709,178 +709,178 @@
     </row>
     <row r="38" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
-        <v>1.4677419350000001</v>
+        <v>0.467741935</v>
       </c>
       <c r="B38" s="2">
-        <v>73.972698359999995</v>
+        <v>-147.5846875</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
-        <v>2.4677419349999998</v>
+        <v>1.4677419350000001</v>
       </c>
       <c r="B39" s="2">
-        <v>69.207098599999995</v>
+        <v>392.72608220000001</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
-        <v>-3.5322580650000002</v>
+        <v>1.4677419350000001</v>
       </c>
       <c r="B40" s="2">
-        <v>-282.54066890000001</v>
+        <v>-215.16667810000001</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
-        <v>-0.53225806499999995</v>
+        <v>1.4677419350000001</v>
       </c>
       <c r="B41" s="2">
-        <v>196.89492379999999</v>
+        <v>-137.25841019999999</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
-        <v>-0.53225806499999995</v>
+        <v>1.4677419350000001</v>
       </c>
       <c r="B42" s="2">
-        <v>-93.904660309999997</v>
+        <v>302.06583760000001</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
-        <v>-2.5322580650000002</v>
+        <v>1.4677419350000001</v>
       </c>
       <c r="B43" s="2">
-        <v>-211.49085249999999</v>
+        <v>383.43439669999998</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
-        <v>-0.53225806499999995</v>
+        <v>1.4677419350000001</v>
       </c>
       <c r="B44" s="2">
-        <v>120.81428390000001</v>
+        <v>85.329523769999994</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
-        <v>-2.5322580650000002</v>
+        <v>1.4677419350000001</v>
       </c>
       <c r="B45" s="2">
-        <v>-101.92164959999999</v>
+        <v>29.76821545</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
-        <v>-0.53225806499999995</v>
+        <v>1.4677419350000001</v>
       </c>
       <c r="B46" s="2">
-        <v>-91.061769920000003</v>
+        <v>86.447454379999996</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
-        <v>-2.5322580650000002</v>
+        <v>1.4677419350000001</v>
       </c>
       <c r="B47" s="2">
-        <v>-201.29575170000001</v>
+        <v>263.80129269999998</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
-        <v>-5.5322580649999997</v>
+        <v>1.4677419350000001</v>
       </c>
       <c r="B48" s="2">
-        <v>-339.99307579999999</v>
+        <v>-10.90527734</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
-        <v>-2.5322580650000002</v>
+        <v>1.4677419350000001</v>
       </c>
       <c r="B49" s="2">
-        <v>-364.66371650000002</v>
+        <v>73.972698359999995</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A50" s="1">
-        <v>-0.53225806499999995</v>
+        <v>1.4677419350000001</v>
       </c>
       <c r="B50" s="2">
-        <v>88.617453889999993</v>
+        <v>155.33541869999999</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A51" s="1">
-        <v>-1.5322580649999999</v>
+        <v>1.4677419350000001</v>
       </c>
       <c r="B51" s="2">
-        <v>-434.67471069999999</v>
+        <v>59.304444519999997</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A52" s="1">
-        <v>-3.5322580650000002</v>
+        <v>2.4677419349999998</v>
       </c>
       <c r="B52" s="2">
-        <v>-177.84190140000001</v>
+        <v>-99.140508990000001</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A53" s="1">
-        <v>-0.53225806499999995</v>
+        <v>2.4677419349999998</v>
       </c>
       <c r="B53" s="2">
-        <v>-59.240526150000001</v>
+        <v>42.346313539999997</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A54" s="1">
-        <v>-1.5322580649999999</v>
+        <v>2.4677419349999998</v>
       </c>
       <c r="B54" s="2">
-        <v>43.387322150000003</v>
+        <v>-14.619110620000001</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A55" s="1">
-        <v>-0.53225806499999995</v>
+        <v>2.4677419349999998</v>
       </c>
       <c r="B55" s="2">
-        <v>99.439455199999998</v>
+        <v>385.94761240000003</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A56" s="1">
-        <v>-1.5322580649999999</v>
+        <v>2.4677419349999998</v>
       </c>
       <c r="B56" s="2">
-        <v>291.83634439999997</v>
+        <v>322.39920560000002</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A57" s="1">
-        <v>-0.53225806499999995</v>
+        <v>2.4677419349999998</v>
       </c>
       <c r="B57" s="2">
-        <v>252.8407685</v>
+        <v>-197.3118254</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A58" s="1">
-        <v>-0.53225806499999995</v>
+        <v>2.4677419349999998</v>
       </c>
       <c r="B58" s="2">
-        <v>426.76154459999998</v>
+        <v>-143.12308340000001</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A59" s="1">
-        <v>1.4677419350000001</v>
+        <v>2.4677419349999998</v>
       </c>
       <c r="B59" s="2">
-        <v>155.33541869999999</v>
+        <v>209.39893910000001</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="21" x14ac:dyDescent="0.3">
@@ -888,37 +888,40 @@
         <v>2.4677419349999998</v>
       </c>
       <c r="B60" s="2">
-        <v>134.23737850000001</v>
+        <v>145.41335430000001</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A61" s="1">
-        <v>-0.53225806499999995</v>
+        <v>2.4677419349999998</v>
       </c>
       <c r="B61" s="2">
-        <v>-157.17071999999999</v>
+        <v>200.7153544</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A62" s="1">
-        <v>1.4677419350000001</v>
+        <v>2.4677419349999998</v>
       </c>
       <c r="B62" s="2">
-        <v>59.304444519999997</v>
+        <v>69.207098599999995</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="21" x14ac:dyDescent="0.3">
       <c r="A63" s="1">
-        <v>0.467741935</v>
+        <v>2.4677419349999998</v>
       </c>
       <c r="B63" s="2">
-        <v>-147.5846875</v>
+        <v>134.23737850000001</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A64" s="1"/>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B64">
+    <sortCondition ref="A2:A64"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>